<commit_message>
UCM model: reprice upside B2 from published UESI booth fees (#21 follow-up)
Upside-only: B2 $8,000 placeholder -> $4,995 published booth + ~$1,500
travel = $6,500 in m14/m26. Re-run engine: upside capital need
$280,023 -> $278,523, ending cash m36 $598,083 -> $601,083; break-even
m19, base and downside byte-identical. Narrowed the §B caveat to the two
items genuinely awaiting HermesX (exhibit-at-all, B4 purchasability) and
documented the B2/B3 registration overlap as assuming a second attendee.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/product/finance/ucm/output/model.xlsx
+++ b/product/finance/ucm/output/model.xlsx
@@ -8658,7 +8658,7 @@
         <v>-250146.71</v>
       </c>
       <c r="C3" s="4">
-        <v>598083.2</v>
+        <v>601083.2</v>
       </c>
       <c r="D3" s="4">
         <v>-740217</v>
@@ -8672,7 +8672,7 @@
         <v>382825.5</v>
       </c>
       <c r="C4" s="4">
-        <v>280022.76</v>
+        <v>278522.76</v>
       </c>
       <c r="D4" s="4">
         <v>740217</v>
@@ -10098,7 +10098,7 @@
         <v>950</v>
       </c>
       <c r="E15" s="5">
-        <f>CHOOSE(MATCH(ScenarioSelector,{"Base","Upside","Downside"},0),147,12346,0)</f>
+        <f>CHOOSE(MATCH(ScenarioSelector,{"Base","Upside","Downside"},0),147,10846,0)</f>
         <v>147</v>
       </c>
       <c r="F15" s="5">

</xml_diff>

<commit_message>
UCM model: reprice upside B2 from published UESI booth fees (#21 follow-up) (#22)
Upside-only: B2 $8,000 placeholder -> $4,995 published booth + ~$1,500
travel = $6,500 in m14/m26. Re-run engine: upside capital need
$280,023 -> $278,523, ending cash m36 $598,083 -> $601,083; break-even
m19, base and downside byte-identical. Narrowed the §B caveat to the two
items genuinely awaiting HermesX (exhibit-at-all, B4 purchasability) and
documented the B2/B3 registration overlap as assuming a second attendee.

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/product/finance/ucm/output/model.xlsx
+++ b/product/finance/ucm/output/model.xlsx
@@ -8658,7 +8658,7 @@
         <v>-250146.71</v>
       </c>
       <c r="C3" s="4">
-        <v>598083.2</v>
+        <v>601083.2</v>
       </c>
       <c r="D3" s="4">
         <v>-740217</v>
@@ -8672,7 +8672,7 @@
         <v>382825.5</v>
       </c>
       <c r="C4" s="4">
-        <v>280022.76</v>
+        <v>278522.76</v>
       </c>
       <c r="D4" s="4">
         <v>740217</v>
@@ -10098,7 +10098,7 @@
         <v>950</v>
       </c>
       <c r="E15" s="5">
-        <f>CHOOSE(MATCH(ScenarioSelector,{"Base","Upside","Downside"},0),147,12346,0)</f>
+        <f>CHOOSE(MATCH(ScenarioSelector,{"Base","Upside","Downside"},0),147,10846,0)</f>
         <v>147</v>
       </c>
       <c r="F15" s="5">

</xml_diff>